<commit_message>
added SLT calibration battery
</commit_message>
<xml_diff>
--- a/data_raw/general_dict.xlsx
+++ b/data_raw/general_dict.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\science\DOTS\development\test_batteries\data_raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\anton_test_batteries\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7135BD-44E6-472F-B302-4A87B17B795C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3E410ED-C0D1-4C34-BFD9-E310ECA98AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3CDF385B-FF42-4ECC-9678-5E042E73A117}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{3CDF385B-FF42-4ECC-9678-5E042E73A117}"/>
   </bookViews>
   <sheets>
     <sheet name="general_dict" sheetId="1" r:id="rId1"/>
@@ -952,10 +952,10 @@
     <t>MPIAE_PROLIFIC_CONSENT_BODY</t>
   </si>
   <si>
-    <t xml:space="preserve">I hereby declare that I have read and understood the information on the study in full. I agree to the described collection and processing of the collected data.  As the data is collected anonymously, it is not possible for me to withdraw my consent at a later date. However, I can cancel my participation at any time by closing the browser window. As a consequence, my data will not be analysed, I cannot be redirected back to Prolific and will therefore not receive any compensation.&lt;br/&gt;In addition, I confirm that I am at least 18 years old and that I am taking part in the study using a device with a keyboard, speakers/headphones and a screen size of at least 11 inches. </t>
-  </si>
-  <si>
     <t>Hiermit erkläre ich, dass ich die Informationen zur Studie vollständig gelesen und verstanden habe. Mit der beschriebenen Erhebung und Verarbeitung der erhobenen Daten bin ich einverstanden.  Da die Daten anonymisiert erhoben werden, ist mein späterer Widerruf der Einwilligung nicht möglich. Ich kann allerdings jederzeit meine Teilnahme beenden, indem ich das Browserfenster schließe. Als Konsequenz werden meine Daten nicht ausgewertet, ich kann nicht zu Prolific zurückgeleitet werden und erhalte daher keine Aufwandsentschädigung. &lt;br/&gt;Zudem bestätige ich, dass ich mindestens 18 Jahre alt bin und mit einem Endgerät mit Tastatur, Lautsprecher/Kopfhörern und einer Bildschirmgröße von mindestens 11 Zoll an der Studie teilnehme.</t>
+  </si>
+  <si>
+    <t>I hereby declare that I have read and understood the information on the study in full. I agree to the described collection and processing of the collected data. \\ As the data is collected anonymously, it is not possible for me to withdraw my consent at a later date. However, I can cancel my participation at any time by closing the browser window. As a consequence, my data will not be analysed, I cannot be redirected back to Prolific and will therefore not receive any compensation. \\ In addition, I confirm that I am at least 18 years old.</t>
   </si>
 </sst>
 </file>
@@ -1099,9 +1099,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1139,7 +1139,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1245,7 +1245,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1387,7 +1387,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1396,14 +1396,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68BC7805-D1BA-4C3B-8218-2DF65AF09233}">
   <dimension ref="A1:C112"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="27.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="41.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="65.85546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="27.1328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="41.73046875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="65.86328125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1425,7 +1425,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>270</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="270" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="213.75" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>30</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>34</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>39</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>48</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>47</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>44</v>
       </c>
@@ -1612,7 +1612,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>49</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>65</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>66</v>
       </c>
@@ -1645,7 +1645,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
         <v>57</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>58</v>
       </c>
@@ -1667,7 +1667,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>61</v>
       </c>
@@ -1678,7 +1678,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>71</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>74</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>77</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>80</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
         <v>85</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
         <v>84</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>86</v>
       </c>
@@ -1755,7 +1755,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="285" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" ht="242.25" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>87</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>83</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
         <v>94</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
         <v>95</v>
       </c>
@@ -1799,7 +1799,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
         <v>99</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>104</v>
       </c>
@@ -1821,7 +1821,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
         <v>108</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>110</v>
       </c>
@@ -1843,7 +1843,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
         <v>109</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
         <v>115</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>118</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>121</v>
       </c>
@@ -1887,7 +1887,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>122</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>128</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="270" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" ht="228" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
         <v>123</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
         <v>67</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
         <v>68</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>134</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>135</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>136</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
         <v>137</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>138</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
         <v>139</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
         <v>140</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
         <v>141</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
         <v>142</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
         <v>143</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" ht="43.15" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A60" s="2" t="s">
         <v>158</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" ht="43.15" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A61" s="2" t="s">
         <v>159</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
         <v>161</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A63" s="2" t="s">
         <v>166</v>
       </c>
@@ -2096,7 +2096,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
         <v>168</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
         <v>169</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
         <v>172</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
         <v>175</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="390" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" ht="313.5" x14ac:dyDescent="0.45">
       <c r="A68" s="2" t="s">
         <v>167</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
         <v>179</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
         <v>183</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
         <v>186</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
         <v>187</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
         <v>194</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
         <v>189</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
         <v>190</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
         <v>191</v>
       </c>
@@ -2239,7 +2239,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
         <v>192</v>
       </c>
@@ -2250,7 +2250,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A78" s="2" t="s">
         <v>193</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A79" s="2" t="s">
         <v>209</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
         <v>212</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
         <v>216</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A82" s="2" t="s">
         <v>217</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A83" s="2" t="s">
         <v>218</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A84" s="2" t="s">
         <v>219</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A85" s="2" t="s">
         <v>220</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A86" s="2" t="s">
         <v>221</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A87" s="2" t="s">
         <v>241</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A88" s="2" t="s">
         <v>242</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A89" s="2" t="s">
         <v>243</v>
       </c>
@@ -2382,7 +2382,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A90" s="2" t="s">
         <v>244</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A91" s="2" t="s">
         <v>245</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A92" s="2" t="s">
         <v>246</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A93" s="2" t="s">
         <v>247</v>
       </c>
@@ -2426,7 +2426,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A94" s="2" t="s">
         <v>248</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A95" s="2" t="s">
         <v>249</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A96" s="2" t="s">
         <v>250</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A97" s="2" t="s">
         <v>254</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A98" s="2" t="s">
         <v>256</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A99" s="2" t="s">
         <v>259</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A100" s="2" t="s">
         <v>260</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A101" s="2" t="s">
         <v>261</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A102" s="2" t="s">
         <v>262</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A103" s="2" t="s">
         <v>267</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="165" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A104" s="2" t="s">
         <v>274</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A105" s="2" t="s">
         <v>275</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A106" s="2" t="s">
         <v>277</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A107" s="2" t="s">
         <v>278</v>
       </c>
@@ -2580,7 +2580,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A108" s="2" t="s">
         <v>291</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="255" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" ht="199.5" x14ac:dyDescent="0.45">
       <c r="A109" s="2" t="s">
         <v>296</v>
       </c>
@@ -2602,7 +2602,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A110" s="2" t="s">
         <v>297</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A111" s="2" t="s">
         <v>298</v>
       </c>
@@ -2624,15 +2624,15 @@
         <v>185</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="285" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" ht="242.25" x14ac:dyDescent="0.45">
       <c r="A112" s="2" t="s">
         <v>307</v>
       </c>
       <c r="B112" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C112" s="2" t="s">
         <v>309</v>
-      </c>
-      <c r="C112" s="2" t="s">
-        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>